<commit_message>
Update latest raw objectives
</commit_message>
<xml_diff>
--- a/latest_raw/futgg_raw_objectives_latest.xlsx
+++ b/latest_raw/futgg_raw_objectives_latest.xlsx
@@ -496,7 +496,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13 03:04:49</t>
+          <t>2026-06-14 03:07:24</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13 02:00:00</t>
+          <t>2026-06-14 02:00:00</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Expires in 7 days</t>
+          <t>Expires in 6 days</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Campaign &gt; Path to Glory Week 2 Path to Glory Week 2 - EA SPORTS FC 26 Objectives Complete all the challenges to earn Festival of Football Tokens and SP. All rewards are Untradeable. NEW Path to Glory Week 2 Complete all the challenges to earn Festival of Football Tokens and SP. All rewards are Untradeable. 20 Tokens Expires in 7 days 800 total 5 Objectives 94% 6% Rewards 800 SP 20 Tokens 15 Tokens 10 Tokens 20 Tokens Goal Getter Score a total of 40 goals in any Ultimate Team Game Mode. 20 Tokens Domination Win 4 games by 3 goals or more in Squad Battles matches on min. Semi-Pro Difficulty (or Live Events/Rivals/Champions/Rush). 300 SP Finesse Glory Score 3 goals with a Finesse Shot in any Ultimate Team Game Mode while having at least 4 players from Australia, Uzbekistan, Qatar or New Zealand in your starting 11. 15 Tokens Path to Glory Win 5 matches in any Ultimate Team Game Mode while having at least 1 Path to Glory or National Pride Player Item in your starting 11. 500 SP The Underdogs Win 6 games in any Ultimate Team Game Mode while having at least 1 Player Item from Saudi Arabia, South Korea and Japan in your starting 11. 10 Tokens © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Campaign &gt; Path to Glory Week 2 Path to Glory Week 2 - EA SPORTS FC 26 Objectives Complete all the challenges to earn Festival of Football Tokens and SP. All rewards are Untradeable. NEW Path to Glory Week 2 Complete all the challenges to earn Festival of Football Tokens and SP. All rewards are Untradeable. 20 Tokens Expires in 6 days 800 total 5 Objectives 93% 7% Rewards 800 SP 20 Tokens 15 Tokens 10 Tokens 20 Tokens Goal Getter Score a total of 40 goals in any Ultimate Team Game Mode. 20 Tokens Domination Win 4 games by 3 goals or more in Squad Battles matches on min. Semi-Pro Difficulty (or Live Events/Rivals/Champions/Rush). 300 SP Finesse Glory Score 3 goals with a Finesse Shot in any Ultimate Team Game Mode while having at least 4 players from Australia, Uzbekistan, Qatar or New Zealand in your starting 11. 15 Tokens Path to Glory Win 5 matches in any Ultimate Team Game Mode while having at least 1 Path to Glory or National Pride Player Item in your starting 11. 500 SP The Underdogs Win 6 games in any Ultimate Team Game Mode while having at least 1 Player Item from Saudi Arabia, South Korea and Japan in your starting 11. 10 Tokens © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -716,7 +716,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Expires in 7 days</t>
+          <t>Expires in 6 days</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Live Events &gt; Journey of Nations Asia &amp; Oceania Journey of Nations Asia &amp; Oceania - EA SPORTS FC 26 Objectives Compete in the Journey of Nations Asia &amp; Oceania Live Event to earn exclusive rewards! All rewards are untradeable. NEW Journey of Nations Asia &amp; Oceania Compete in the Journey of Nations Asia &amp; Oceania Live Event to earn exclusive rewards! All rewards are untradeable. 87+ Rare Gold Player Pack Expires in 7 days 6 Objectives 87% 13% Rewards Shadow Award Hunter 1x 2x 84+ Rare Gold Players Pack 1x 5x 81+ Rare Gold Players Pack 1x 5x 80+ Rare Gold Players Pack 1x 87+ Rare Gold Player Pack Win 3 Win 3 matches in the Journey of Nations Asia &amp; Oceania Live Event. Shadow Play 3 Play 3 matches in the Journey of Nations Asia &amp; Oceania Live Event. Award Win 2 Win 2 matches in the Journey of Nations Asia &amp; Oceania Live Event. 2X 84+ Rare Gold Players Pack Play 2 Play 2 matches in the Journey of Nations Asia &amp; Oceania Live Event. 5X 81+ Rare Gold Players Pack Win 1 Win 1 match in the Journey of Nations Asia &amp; Oceania Live Event. 5X 80+ Rare Gold Players Pack Play 1 Play 1 match in the Journey of Nations Asia &amp; Oceania Live Event. Hunter © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Live Events &gt; Journey of Nations Asia &amp; Oceania Journey of Nations Asia &amp; Oceania - EA SPORTS FC 26 Objectives Compete in the Journey of Nations Asia &amp; Oceania Live Event to earn exclusive rewards! All rewards are untradeable. NEW Journey of Nations Asia &amp; Oceania Compete in the Journey of Nations Asia &amp; Oceania Live Event to earn exclusive rewards! All rewards are untradeable. 87+ Rare Gold Player Pack Expires in 6 days 6 Objectives 90% 10% Rewards Shadow Award Hunter 1x 2x 84+ Rare Gold Players Pack 1x 5x 81+ Rare Gold Players Pack 1x 5x 80+ Rare Gold Players Pack 1x 87+ Rare Gold Player Pack Win 3 Win 3 matches in the Journey of Nations Asia &amp; Oceania Live Event. Shadow Play 3 Play 3 matches in the Journey of Nations Asia &amp; Oceania Live Event. Award Win 2 Win 2 matches in the Journey of Nations Asia &amp; Oceania Live Event. 2X 84+ Rare Gold Players Pack Play 2 Play 2 matches in the Journey of Nations Asia &amp; Oceania Live Event. 5X 81+ Rare Gold Players Pack Win 1 Win 1 match in the Journey of Nations Asia &amp; Oceania Live Event. 5X 80+ Rare Gold Players Pack Play 1 Play 1 match in the Journey of Nations Asia &amp; Oceania Live Event. Hunter © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Campaign &gt; Weekly Rush Points Weekly Rush Points - EA SPORTS FC 26 Objectives Complete Rush Bonuses alongside your teammates to earn Rush Points! Weekly Rush Points Complete Rush Bonuses alongside your teammates to earn Rush Points! 2X 89+ Rare Gold Players Pack 100 Tokens Expires in 6 days 5 Objectives 79% 21% Rewards 100 Tokens 1x 88+ Rare Gold Player Pack 1x 2x 85+ Rare Gold Players Pack 1x 4x 84+ Rare Gold Players Pack 1x 3x 84+ Rare Gold Players Pack 1x 4x 83+ Rare Gold Players Pack 1x 2x 89+ Rare Gold Players Pack 45,000 Rush Points Earn 45,000 points by completing bonuses in Rush. 88+ Rare Gold Player Pack 35,000 Rush Points Earn 35,000 points by completing bonuses in Rush. 2X 85+ Rare Gold Players Pack 25,000 Rush Points Earn 25,000 points by completing bonuses in Rush. 4X 84+ Rare Gold Players Pack 10,000 Rush Points Earn 10,000 points by completing bonuses in Rush. 3X 84+ Rare Gold Players Pack 2,500 Rush Points Earn 2,500 points by completing bonuses in Rush. 4X 83+ Rare Gold Players Pack © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Campaign &gt; Weekly Rush Points Weekly Rush Points - EA SPORTS FC 26 Objectives Complete Rush Bonuses alongside your teammates to earn Rush Points! Weekly Rush Points Complete Rush Bonuses alongside your teammates to earn Rush Points! 2X 89+ Rare Gold Players Pack 100 Tokens Expires in 5 days 5 Objectives 79% 21% Rewards 100 Tokens 1x 88+ Rare Gold Player Pack 1x 2x 85+ Rare Gold Players Pack 1x 4x 84+ Rare Gold Players Pack 1x 3x 84+ Rare Gold Players Pack 1x 4x 83+ Rare Gold Players Pack 1x 2x 89+ Rare Gold Players Pack 45,000 Rush Points Earn 45,000 points by completing bonuses in Rush. 88+ Rare Gold Player Pack 35,000 Rush Points Earn 35,000 points by completing bonuses in Rush. 2X 85+ Rare Gold Players Pack 25,000 Rush Points Earn 25,000 points by completing bonuses in Rush. 4X 84+ Rare Gold Players Pack 10,000 Rush Points Earn 10,000 points by completing bonuses in Rush. 3X 84+ Rare Gold Players Pack 2,500 Rush Points Earn 2,500 points by completing bonuses in Rush. 4X 83+ Rare Gold Players Pack © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Seasonal &gt; Season 8 Weekly Play 2 Season 8 Weekly Play 2 - EA SPORTS FC 26 Objectives Complete 3 out of the 5 challenges to earn SP! Season 8 Weekly Play 2 Complete 3 out of the 5 challenges to earn SP! 750 SP Expires in 6 days 2,000 total 3 of 5 Objectives 94% 6% Rewards 2,000 SP Play 5 Live Events Play 5 matches in any Ultimate Team Live Event. 250 SP Play 5 Rush Play 5 Ultimate Team Rush matches. 250 SP Play 5 Champions Play 5 matches in Champions. 250 SP Play 5 Rivals Play 5 matches in Rivals. 250 SP Play 5 Squad Battles Play 5 Squad Battles matches on Min. Semi-Pro difficulty. 250 SP © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Seasonal &gt; Season 8 Weekly Play 2 Season 8 Weekly Play 2 - EA SPORTS FC 26 Objectives Complete 3 out of the 5 challenges to earn SP! Season 8 Weekly Play 2 Complete 3 out of the 5 challenges to earn SP! 750 SP Expires in 5 days 2,000 total 3 of 5 Objectives 94% 6% Rewards 2,000 SP Play 5 Live Events Play 5 matches in any Ultimate Team Live Event. 250 SP Play 5 Rush Play 5 Ultimate Team Rush matches. 250 SP Play 5 Champions Play 5 matches in Champions. 250 SP Play 5 Rivals Play 5 matches in Rivals. 250 SP Play 5 Squad Battles Play 5 Squad Battles matches on Min. Semi-Pro difficulty. 250 SP © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -866,7 +866,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -881,7 +881,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Seasonal &gt; Weekly Objectives Weekly Objectives - EA SPORTS FC 26 Objectives Complete weekly Objectives to earn SP! Weekly Objectives Complete weekly Objectives to earn SP! 500 SP Expires in 6 days 1,500 total 5 Objectives 95% 5% Rewards 1,500 SP Score 10 Score 10 goals in any Ultimate Team game mode using a player from Canada. 200 SP Win 10 Win 10 matches in Squad Battles on Min. Semi-Pro difficulty (or Rush/Rivals/Champions/Live Events). 200 SP Play 10 Play 10 matches in Squad Battles on Min. Semi-Pro difficulty (or Rush/Rivals/Champions/Live Events). 200 SP Buy 10 Buy 10 Player Items on the Transfer Market. 200 SP List 10 List 10 Player Items on the Transfer Market. 200 SP © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Seasonal &gt; Weekly Objectives Weekly Objectives - EA SPORTS FC 26 Objectives Complete weekly Objectives to earn SP! Weekly Objectives Complete weekly Objectives to earn SP! 500 SP Expires in 5 days 1,500 total 5 Objectives 96% 4% Rewards 1,500 SP Score 10 Score 10 goals in any Ultimate Team game mode using a player from Canada. 200 SP Win 10 Win 10 matches in Squad Battles on Min. Semi-Pro difficulty (or Rush/Rivals/Champions/Live Events). 200 SP Play 10 Play 10 matches in Squad Battles on Min. Semi-Pro difficulty (or Rush/Rivals/Champions/Live Events). 200 SP Buy 10 Buy 10 Player Items on the Transfer Market. 200 SP List 10 List 10 Player Items on the Transfer Market. 200 SP © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -916,22 +916,22 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Expires in 2 days</t>
+          <t>Expires in 23 hours</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>6/15 02:00</t>
+          <t>6/15 01:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15T02:00+09:00</t>
+          <t>2026-06-15T01:00+09:00</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Live Events &gt; Path to Glory! Path to Glory! - EA SPORTS FC 26 Objectives Celebrate some of the week's standout international matches in the Path to Glory Live Event with this themed Objective! Earn packs, FOF Tokens, SP, one celebration item, and EVO Rewards. All rewards are untradeable. Path to Glory! Celebrate some of the week's standout international matches in the Path to Glory Live Event with this themed Objective! Earn packs, FOF Tokens, SP, one celebration item, and EVO Rewards. All rewards are untradeable. 170 Tokens Evo Unlock Expires in 2 days 500 total 9 Objectives 86% 14% Rewards 500 SP 90 Tokens Award Evo Unlock 40 Tokens Evo Unlock 170 Tokens Evo Unlock 1x 3x 84+ Rare Gold Players Pack 1x 3x 86+ Rare Gold Players Pack 1x 4x 85+ Rare Gold Players Pack 1x 7x 84+ Rare Gold Players Pack 1x 7x 82+ Rare Gold Players Pack 1x 10x 81+ Rare Gold Players Pack Brazil vs. Morocco Assist 5 goals in the Path to Glory Live Event while having min. 4 players from Brazil or Morocco in your starting 11. 500 SP Qatar vs. Switzerland Win 3 matches in the Path to Glory Live Event while having min. 4 players from Qatar or Switzerland in your starting 11. 90 Tokens 3X 84+ Rare Gold Players Pack Austria vs. Türkiye Score 5 goals in the Path to Glory Live Event while having min. 4 players from Austria or Turkiye in your starting 11. 3X 86+ Rare Gold Players Pack Canada vs. Bosnia and Herzegovina Win 2 matches in the Path to Glory Live Event while having min. 4 players from Canada or Bosnia and Herzegovina in your starting 11. 4X 85+ Rare Gold Players Pack United States vs. Paraguay Play 2 matches in the Path to Glory Live Event while having min. 4 players from USA or Paraguay in your starting 11. 7X 84+ Rare Gold Players Pack Mexico vs. South Africa Score 3 goals in the Path to Glory Live Event while having min. 4 players from Mexico or South Africa in your starting 11. Award South Korea vs. Czechia Score 2 goals with Finesse Shots in the Path to Glory Live Event while having min. 4 players from South Korea or Czechia in your starting 11. Earn an Evo consumable. All EVO details can be previewed. Evo Unlock Score 10 Score 10 goals in the Path to Glory Live Event. 40 Tokens 7X 82+ Rare Gold Players Pack Score 1 Score 1 goal in the Path to Glory Live Event. Earn a Cosmetic EVO. All EVO details can be previewed. Evo Unlock 10X 81+ Rare Gold Players Pack © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Live Events &gt; Path to Glory! Path to Glory! - EA SPORTS FC 26 Objectives Celebrate some of the week's standout international matches in the Path to Glory Live Event with this themed Objective! Earn packs, FOF Tokens, SP, one celebration item, and EVO Rewards. All rewards are untradeable. Path to Glory! Celebrate some of the week's standout international matches in the Path to Glory Live Event with this themed Objective! Earn packs, FOF Tokens, SP, one celebration item, and EVO Rewards. All rewards are untradeable. 170 Tokens Evo Unlock Expires in 23 hours 500 total 9 Objectives 86% 14% Rewards 500 SP 90 Tokens Award Evo Unlock 40 Tokens Evo Unlock 170 Tokens Evo Unlock 1x 3x 84+ Rare Gold Players Pack 1x 3x 86+ Rare Gold Players Pack 1x 4x 85+ Rare Gold Players Pack 1x 7x 84+ Rare Gold Players Pack 1x 7x 82+ Rare Gold Players Pack 1x 10x 81+ Rare Gold Players Pack Brazil vs. Morocco Assist 5 goals in the Path to Glory Live Event while having min. 4 players from Brazil or Morocco in your starting 11. 500 SP Qatar vs. Switzerland Win 3 matches in the Path to Glory Live Event while having min. 4 players from Qatar or Switzerland in your starting 11. 90 Tokens 3X 84+ Rare Gold Players Pack Austria vs. Türkiye Score 5 goals in the Path to Glory Live Event while having min. 4 players from Austria or Turkiye in your starting 11. 3X 86+ Rare Gold Players Pack Canada vs. Bosnia and Herzegovina Win 2 matches in the Path to Glory Live Event while having min. 4 players from Canada or Bosnia and Herzegovina in your starting 11. 4X 85+ Rare Gold Players Pack United States vs. Paraguay Play 2 matches in the Path to Glory Live Event while having min. 4 players from USA or Paraguay in your starting 11. 7X 84+ Rare Gold Players Pack Mexico vs. South Africa Score 3 goals in the Path to Glory Live Event while having min. 4 players from Mexico or South Africa in your starting 11. Award South Korea vs. Czechia Score 2 goals with Finesse Shots in the Path to Glory Live Event while having min. 4 players from South Korea or Czechia in your starting 11. Earn an Evo consumable. All EVO details can be previewed. Evo Unlock Score 10 Score 10 goals in the Path to Glory Live Event. 40 Tokens 7X 82+ Rare Gold Players Pack Score 1 Score 1 goal in the Path to Glory Live Event. Earn a Cosmetic EVO. All EVO details can be previewed. Evo Unlock 10X 81+ Rare Gold Players Pack © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -981,7 +981,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Seasonal &gt; Daily Objectives Daily Objectives - EA SPORTS FC 26 Objectives Play, complete, and earn SP from the daily Objective every 24 hours! Daily Objectives Play, complete, and earn SP from the daily Objective every 24 hours! 90 SP Expires in 6 days 190 total 2 Objectives 92% 8% Rewards 190 SP Score 2 goals Score 2 goals in any Ultimate Team game mode. 50 SP Play 1 Play 1 match in any Ultimate Team game mode and earn SP! 50 SP © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Seasonal &gt; Daily Objectives Daily Objectives - EA SPORTS FC 26 Objectives Play, complete, and earn SP from the daily Objective every 24 hours! Daily Objectives Play, complete, and earn SP from the daily Objective every 24 hours! 90 SP Expires in 5 days 190 total 2 Objectives 92% 8% Rewards 190 SP Score 2 goals Score 2 goals in any Ultimate Team game mode. 50 SP Play 1 Play 1 match in any Ultimate Team game mode and earn SP! 50 SP © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Seasonal &gt; Season 8 Weekly Play Completionist Season 8 Weekly Play Completionist - EA SPORTS FC 26 Objectives Complete any 4 of the 5 Season 8 Weekly Play Objectives and claim bonus pack rewards. All rewards are untradeable. Season 8 Weekly Play Completionist Complete any 4 of the 5 Season 8 Weekly Play Objectives and claim bonus pack rewards. All rewards are untradeable. Fof Ptg Player Pack Expires in 27 days 4 of 5 Objectives 91% 9% Rewards 1 Of 4 89+ Rare Gold Player Pick 1 Of 4 89+ Rare Gold Player Pick 1x 5x 88+ Rare Gold Players Pack 1x 3x 85+ Rare Gold Players Pack 1x 4x 84+ Rare Gold Players Pack 1x FOF PTG Player Pack Week 5 Complete the Season 8 Weekly Play 5 Objective. 1 Of 4 89+ Rare Gold Player Pick Week 4 Complete the Season 8 Weekly Play 4 Objective. 1 Of 4 89+ Rare Gold Player Pick Week 3 Complete the Season 8 Weekly Play 3 Objective. 5X 88+ Rare Gold Players Pack Week 2 Complete the Season 8 Weekly Play 2 Objective. 3X 85+ Rare Gold Players Pack Week 1 Complete the Season 8 Weekly Play 1 Objective. 4X 84+ Rare Gold Players Pack © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Seasonal &gt; Season 8 Weekly Play Completionist Season 8 Weekly Play Completionist - EA SPORTS FC 26 Objectives Complete any 4 of the 5 Season 8 Weekly Play Objectives and claim bonus pack rewards. All rewards are untradeable. Season 8 Weekly Play Completionist Complete any 4 of the 5 Season 8 Weekly Play Objectives and claim bonus pack rewards. All rewards are untradeable. Fof Ptg Player Pack Expires in 26 days 4 of 5 Objectives 91% 9% Rewards 1 Of 4 89+ Rare Gold Player Pick 1 Of 4 89+ Rare Gold Player Pick 1x 5x 88+ Rare Gold Players Pack 1x 3x 85+ Rare Gold Players Pack 1x 4x 84+ Rare Gold Players Pack 1x FOF PTG Player Pack Week 5 Complete the Season 8 Weekly Play 5 Objective. 1 Of 4 89+ Rare Gold Player Pick Week 4 Complete the Season 8 Weekly Play 4 Objective. 1 Of 4 89+ Rare Gold Player Pick Week 3 Complete the Season 8 Weekly Play 3 Objective. 5X 88+ Rare Gold Players Pack Week 2 Complete the Season 8 Weekly Play 2 Objective. 3X 85+ Rare Gold Players Pack Week 1 Complete the Season 8 Weekly Play 1 Objective. 4X 84+ Rare Gold Players Pack © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Live Events &gt; Season 8 Exhibition Weekly Play Completionist Season 8 Exhibition Weekly Play Completionist - EA SPORTS FC 26 Objectives Compete in the Season 8 Exhibition event to earn exclusive rewards! All rewards are untradeable. Season 8 Exhibition Weekly Play Completionist Compete in the Season 8 Exhibition event to earn exclusive rewards! All rewards are untradeable. 1 Of 3 94+ Fof Ptg/Gotg/Gh Team 1 Player Pick Expires in 27 days 5 Objectives 89% 11% Rewards 1 Of 3 Fof Gh Team 1 Player Pick 1 Of 3 Fof Gotg Player Pick 1 Of 3 94+ Fof Ptg/Gotg/Gh Team 1 Player Pick 1x 93+ FOF PTG Team 2 Player Pack 1x 93+ FOF PTG Team 1 Player Pack 1x 5x 87+ Rare Gold Players Pack Week 5 Complete the Season 8 Exhibition Weekly Play Objective 5 times. 1 Of 3 Fof Gh Team 1 Player Pick Week 4 Complete the Season 8 Exhibition Weekly Play Objective 4 times. 1 Of 3 Fof Gotg Player Pick Week 3 Complete the Season 8 Exhibition Weekly Play Objective 3 times. 93+ Fof Ptg Team 2 Player Pack Week 2 Complete the Season 8 Exhibition Weekly Play Objective 2 times. 93+ Fof Ptg Team 1 Player Pack Week 1 Complete the Season 8 Exhibition Weekly Play Objective 1 time. 5X 87+ Rare Gold Players Pack © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Live Events &gt; Season 8 Exhibition Weekly Play Completionist Season 8 Exhibition Weekly Play Completionist - EA SPORTS FC 26 Objectives Compete in the Season 8 Exhibition event to earn exclusive rewards! All rewards are untradeable. Season 8 Exhibition Weekly Play Completionist Compete in the Season 8 Exhibition event to earn exclusive rewards! All rewards are untradeable. 1 Of 3 94+ Fof Ptg/Gotg/Gh Team 1 Player Pick Expires in 26 days 5 Objectives 89% 11% Rewards 1 Of 3 Fof Gh Team 1 Player Pick 1 Of 3 Fof Gotg Player Pick 1 Of 3 94+ Fof Ptg/Gotg/Gh Team 1 Player Pick 1x 93+ FOF PTG Team 2 Player Pack 1x 93+ FOF PTG Team 1 Player Pack 1x 5x 87+ Rare Gold Players Pack Week 5 Complete the Season 8 Exhibition Weekly Play Objective 5 times. 1 Of 3 Fof Gh Team 1 Player Pick Week 4 Complete the Season 8 Exhibition Weekly Play Objective 4 times. 1 Of 3 Fof Gotg Player Pick Week 3 Complete the Season 8 Exhibition Weekly Play Objective 3 times. 93+ Fof Ptg Team 2 Player Pack Week 2 Complete the Season 8 Exhibition Weekly Play Objective 2 times. 93+ Fof Ptg Team 1 Player Pack Week 1 Complete the Season 8 Exhibition Weekly Play Objective 1 time. 5X 87+ Rare Gold Players Pack © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Live Events &gt; Season 8 Exhibition Weekly Play Season 8 Exhibition Weekly Play - EA SPORTS FC 26 Objectives Compete in the Season 8 Exhibition event to earn Coin boost and a consumable item! All rewards are untradeable. Season 8 Exhibition Weekly Play Compete in the Season 8 Exhibition event to earn Coin boost and a consumable item! All rewards are untradeable. Shadow Expires in 27 days 1 Objectives 91% 9% Rewards Item Shadow Play 9 Play 9 matches in the Season 8 Exhibition event. Item © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Live Events &gt; Season 8 Exhibition Weekly Play Season 8 Exhibition Weekly Play - EA SPORTS FC 26 Objectives Compete in the Season 8 Exhibition event to earn Coin boost and a consumable item! All rewards are untradeable. Season 8 Exhibition Weekly Play Compete in the Season 8 Exhibition event to earn Coin boost and a consumable item! All rewards are untradeable. Shadow Expires in 26 days 1 Objectives 91% 9% Rewards Item Shadow Play 9 Play 9 matches in the Season 8 Exhibition event. Item © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Live Events &gt; Season 8 Exhibition Season 8 Exhibition - EA SPORTS FC 26 Objectives Compete in the Season 8 Exhibition event to earn exclusive rewards! All rewards are untradeable. Season 8 Exhibition Compete in the Season 8 Exhibition event to earn exclusive rewards! All rewards are untradeable. 5X 88+ Rare Gold Players Pack Evo Unlock Expires in 27 days 7 Objectives 90% 10% Rewards Evo Unlock Evo Unlock 1 Of 4 89+ Rare Gold Player Pick 1 Of 4 88+ Rare Gold Players Evo Unlock 1x 10x 87+ Rare Gold Players Pack 1x 5x 87+ Rare Gold Players Pack 1x 3x 88+ Rare Gold Players Pack 1x 5x 88+ Rare Gold Players Pack Score in 30 Score at least 1 goal in 30 separate matches in the Season 8 Exhibition event. Evo Unlock Score in 25 Score at least 1 goal in 25 separate matches in the Season 8 Exhibition event. Evo Unlock Score in 20 Score at least 1 goal in 20 separate matches with a ST in the Season 8 Exhibition event. 10X 87+ Rare Gold Players Pack Assist in 20 Assist at least 1 goal in 20 separate matches with a CM in the Season 8 Exhibition event. 1 Of 4 89+ Rare Gold Player Pick Play 20 Play 20 matches in the Season 8 Exhibition event. 5X 87+ Rare Gold Players Pack Play 10 Play 10 matches in the Season 8 Exhibition event. 1 Of 4 88+ Rare Gold Players Play 5 Play 5 matches in the Season 8 Exhibition event. 3X 88+ Rare Gold Players Pack © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Live Events &gt; Season 8 Exhibition Season 8 Exhibition - EA SPORTS FC 26 Objectives Compete in the Season 8 Exhibition event to earn exclusive rewards! All rewards are untradeable. Season 8 Exhibition Compete in the Season 8 Exhibition event to earn exclusive rewards! All rewards are untradeable. 5X 88+ Rare Gold Players Pack Evo Unlock Expires in 26 days 7 Objectives 90% 10% Rewards Evo Unlock Evo Unlock 1 Of 4 89+ Rare Gold Player Pick 1 Of 4 88+ Rare Gold Players Evo Unlock 1x 10x 87+ Rare Gold Players Pack 1x 5x 87+ Rare Gold Players Pack 1x 3x 88+ Rare Gold Players Pack 1x 5x 88+ Rare Gold Players Pack Score in 30 Score at least 1 goal in 30 separate matches in the Season 8 Exhibition event. Evo Unlock Score in 25 Score at least 1 goal in 25 separate matches in the Season 8 Exhibition event. Evo Unlock Score in 20 Score at least 1 goal in 20 separate matches with a ST in the Season 8 Exhibition event. 10X 87+ Rare Gold Players Pack Assist in 20 Assist at least 1 goal in 20 separate matches with a CM in the Season 8 Exhibition event. 1 Of 4 89+ Rare Gold Player Pick Play 20 Play 20 matches in the Season 8 Exhibition event. 5X 87+ Rare Gold Players Pack Play 10 Play 10 matches in the Season 8 Exhibition event. 1 Of 4 88+ Rare Gold Players Play 5 Play 5 matches in the Season 8 Exhibition event. 3X 88+ Rare Gold Players Pack © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -2666,7 +2666,7 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>Expires in 7 days</t>
+          <t>Expires in 6 days</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
@@ -2746,7 +2746,7 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>Expires in 7 days</t>
+          <t>Expires in 6 days</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>Expires in 7 days</t>
+          <t>Expires in 6 days</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
@@ -2898,7 +2898,7 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>Expires in 7 days</t>
+          <t>Expires in 6 days</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
@@ -2974,7 +2974,7 @@
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>Expires in 7 days</t>
+          <t>Expires in 6 days</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>Expires in 7 days</t>
+          <t>Expires in 6 days</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
@@ -3126,7 +3126,7 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>Expires in 7 days</t>
+          <t>Expires in 6 days</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
@@ -3202,7 +3202,7 @@
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>Expires in 7 days</t>
+          <t>Expires in 6 days</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
@@ -3278,7 +3278,7 @@
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>Expires in 7 days</t>
+          <t>Expires in 6 days</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>Expires in 7 days</t>
+          <t>Expires in 6 days</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
@@ -3430,7 +3430,7 @@
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>Expires in 7 days</t>
+          <t>Expires in 6 days</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr">
@@ -3582,7 +3582,7 @@
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
@@ -3658,7 +3658,7 @@
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
@@ -3734,7 +3734,7 @@
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
@@ -3810,7 +3810,7 @@
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
@@ -3886,7 +3886,7 @@
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
@@ -3962,7 +3962,7 @@
       </c>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M19" s="3" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M21" s="3" t="inlineStr">
@@ -4190,7 +4190,7 @@
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr">
@@ -4266,7 +4266,7 @@
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr">
@@ -4342,7 +4342,7 @@
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M24" s="3" t="inlineStr">
@@ -4418,7 +4418,7 @@
       </c>
       <c r="L25" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M25" s="3" t="inlineStr">
@@ -4494,7 +4494,7 @@
       </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M26" s="3" t="inlineStr">
@@ -4570,7 +4570,7 @@
       </c>
       <c r="L27" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M27" s="3" t="inlineStr">
@@ -4650,7 +4650,7 @@
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M28" s="3" t="inlineStr">
@@ -4726,7 +4726,7 @@
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M29" s="3" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M30" s="3" t="inlineStr">
@@ -4886,7 +4886,7 @@
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr">
@@ -4962,17 +4962,17 @@
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>Expires in 2 days</t>
+          <t>Expires in 23 hours</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>6/15 02:00</t>
+          <t>6/15 01:00</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15T02:00+09:00</t>
+          <t>2026-06-15T01:00+09:00</t>
         </is>
       </c>
       <c r="O32" s="2" t="inlineStr">
@@ -5038,17 +5038,17 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Expires in 2 days</t>
+          <t>Expires in 23 hours</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>6/15 02:00</t>
+          <t>6/15 01:00</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15T02:00+09:00</t>
+          <t>2026-06-15T01:00+09:00</t>
         </is>
       </c>
       <c r="O33" s="2" t="inlineStr">
@@ -5114,17 +5114,17 @@
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>Expires in 2 days</t>
+          <t>Expires in 23 hours</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>6/15 02:00</t>
+          <t>6/15 01:00</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15T02:00+09:00</t>
+          <t>2026-06-15T01:00+09:00</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
@@ -5190,17 +5190,17 @@
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>Expires in 2 days</t>
+          <t>Expires in 23 hours</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>6/15 02:00</t>
+          <t>6/15 01:00</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15T02:00+09:00</t>
+          <t>2026-06-15T01:00+09:00</t>
         </is>
       </c>
       <c r="O35" s="2" t="inlineStr">
@@ -5266,17 +5266,17 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>Expires in 2 days</t>
+          <t>Expires in 23 hours</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>6/15 02:00</t>
+          <t>6/15 01:00</t>
         </is>
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15T02:00+09:00</t>
+          <t>2026-06-15T01:00+09:00</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr">
@@ -5342,17 +5342,17 @@
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>Expires in 2 days</t>
+          <t>Expires in 23 hours</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>6/15 02:00</t>
+          <t>6/15 01:00</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15T02:00+09:00</t>
+          <t>2026-06-15T01:00+09:00</t>
         </is>
       </c>
       <c r="O37" s="2" t="inlineStr">
@@ -5418,17 +5418,17 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>Expires in 2 days</t>
+          <t>Expires in 23 hours</t>
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>6/15 02:00</t>
+          <t>6/15 01:00</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15T02:00+09:00</t>
+          <t>2026-06-15T01:00+09:00</t>
         </is>
       </c>
       <c r="O38" s="2" t="inlineStr">
@@ -5494,17 +5494,17 @@
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>Expires in 2 days</t>
+          <t>Expires in 23 hours</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>6/15 02:00</t>
+          <t>6/15 01:00</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15T02:00+09:00</t>
+          <t>2026-06-15T01:00+09:00</t>
         </is>
       </c>
       <c r="O39" s="2" t="inlineStr">
@@ -5570,17 +5570,17 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>Expires in 2 days</t>
+          <t>Expires in 23 hours</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>6/15 02:00</t>
+          <t>6/15 01:00</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15T02:00+09:00</t>
+          <t>2026-06-15T01:00+09:00</t>
         </is>
       </c>
       <c r="O40" s="2" t="inlineStr">
@@ -5642,7 +5642,7 @@
       </c>
       <c r="L41" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M41" s="3" t="inlineStr">
@@ -5718,7 +5718,7 @@
       </c>
       <c r="L42" s="3" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M42" s="3" t="inlineStr">
@@ -5794,7 +5794,7 @@
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="M43" s="2" t="inlineStr">
@@ -5866,7 +5866,7 @@
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="M44" s="2" t="inlineStr">
@@ -5938,7 +5938,7 @@
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="M45" s="2" t="inlineStr">
@@ -6010,7 +6010,7 @@
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="M46" s="2" t="inlineStr">
@@ -6082,7 +6082,7 @@
       </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="M47" s="2" t="inlineStr">
@@ -6154,7 +6154,7 @@
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr">
@@ -6226,7 +6226,7 @@
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="M49" s="2" t="inlineStr">
@@ -6298,7 +6298,7 @@
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="M50" s="2" t="inlineStr">
@@ -6370,7 +6370,7 @@
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="M51" s="2" t="inlineStr">
@@ -6442,7 +6442,7 @@
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="M52" s="2" t="inlineStr">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="M53" s="2" t="inlineStr">
@@ -6586,7 +6586,7 @@
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="M54" s="2" t="inlineStr">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="M55" s="2" t="inlineStr">
@@ -6738,7 +6738,7 @@
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="M56" s="2" t="inlineStr">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="M57" s="2" t="inlineStr">
@@ -6890,7 +6890,7 @@
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="M58" s="2" t="inlineStr">
@@ -6966,7 +6966,7 @@
       </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="M59" s="2" t="inlineStr">
@@ -7042,7 +7042,7 @@
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="M60" s="2" t="inlineStr">
@@ -7118,7 +7118,7 @@
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="M61" s="2" t="inlineStr">
@@ -17241,12 +17241,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>NEW Path to Glory Week 2 Complete all the challenges to earn Festival of Football Tokens and SP. All rewards are Untradeable. 20 Tokens Expires in 7 days 800 total 5 Objectives 94% 6%</t>
+          <t>NEW Path to Glory Week 2 Complete all the challenges to earn Festival of Football Tokens and SP. All rewards are Untradeable. 20 Tokens Expires in 6 days 800 total 5 Objectives 93% 7%</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Expires in 7 days</t>
+          <t>Expires in 6 days</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -17278,12 +17278,12 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>NEW Journey of Nations Asia &amp; Oceania Compete in the Journey of Nations Asia &amp; Oceania Live Event to earn exclusive rewards! All rewards are untradeable. 87+ Rare Gold Player Pack Expires in 7 days 6 Objectives 87% 13%</t>
+          <t>NEW Journey of Nations Asia &amp; Oceania Compete in the Journey of Nations Asia &amp; Oceania Live Event to earn exclusive rewards! All rewards are untradeable. 87+ Rare Gold Player Pack Expires in 6 days 6 Objectives 90% 10%</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Expires in 7 days</t>
+          <t>Expires in 6 days</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -17315,12 +17315,12 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Weekly Rush Points Complete Rush Bonuses alongside your teammates to earn Rush Points! 2X 89+ Rare Gold Players Pack 100 Tokens Expires in 6 days 5 Objectives 79% 21%</t>
+          <t>Weekly Rush Points Complete Rush Bonuses alongside your teammates to earn Rush Points! 2X 89+ Rare Gold Players Pack 100 Tokens Expires in 5 days 5 Objectives 79% 21%</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -17352,12 +17352,12 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Season 8 Weekly Play 2 Complete 3 out of the 5 challenges to earn SP! 750 SP Expires in 6 days 2,000 total 3 of 5 Objectives 94% 6%</t>
+          <t>Season 8 Weekly Play 2 Complete 3 out of the 5 challenges to earn SP! 750 SP Expires in 5 days 2,000 total 3 of 5 Objectives 94% 6%</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -17389,12 +17389,12 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Weekly Objectives Complete weekly Objectives to earn SP! 500 SP Expires in 6 days 1,500 total 5 Objectives 95% 5%</t>
+          <t>Weekly Objectives Complete weekly Objectives to earn SP! 500 SP Expires in 5 days 1,500 total 5 Objectives 96% 4%</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -17426,22 +17426,22 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Path to Glory! Celebrate some of the week's standout international matches in the Path to Glory Live Event with this themed Objective! Earn packs, FOF Tokens, SP, one celebration item, and EVO Rewards. All rewards are untradeable. 170 Tokens Evo Unlock Expires in 2 days 500 total 9 Objectives 86% 14%</t>
+          <t>Path to Glory! Celebrate some of the week's standout international matches in the Path to Glory Live Event with this themed Objective! Earn packs, FOF Tokens, SP, one celebration item, and EVO Rewards. All rewards are untradeable. 170 Tokens Evo Unlock Expires in 23 hours 500 total 9 Objectives 86% 14%</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Expires in 2 days</t>
+          <t>Expires in 23 hours</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>6/15 02:00</t>
+          <t>6/15 01:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15T02:00+09:00</t>
+          <t>2026-06-15T01:00+09:00</t>
         </is>
       </c>
     </row>
@@ -17463,12 +17463,12 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Daily Objectives Play, complete, and earn SP from the daily Objective every 24 hours! 90 SP Expires in 6 days 190 total 2 Objectives 92% 8%</t>
+          <t>Daily Objectives Play, complete, and earn SP from the daily Objective every 24 hours! 90 SP Expires in 5 days 190 total 2 Objectives 92% 8%</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Expires in 6 days</t>
+          <t>Expires in 5 days</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -17500,12 +17500,12 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Season 8 Weekly Play Completionist Complete any 4 of the 5 Season 8 Weekly Play Objectives and claim bonus pack rewards. All rewards are untradeable. Fof Ptg Player Pack Expires in 27 days 4 of 5 Objectives 91% 9%</t>
+          <t>Season 8 Weekly Play Completionist Complete any 4 of the 5 Season 8 Weekly Play Objectives and claim bonus pack rewards. All rewards are untradeable. Fof Ptg Player Pack Expires in 26 days 4 of 5 Objectives 91% 9%</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -17537,12 +17537,12 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Season 8 Exhibition Weekly Play Completionist Compete in the Season 8 Exhibition event to earn exclusive rewards! All rewards are untradeable. 1 Of 3 94+ Fof Ptg/Gotg/Gh Team 1 Player Pick Expires in 27 days 5 Objectives 89% 11%</t>
+          <t>Season 8 Exhibition Weekly Play Completionist Compete in the Season 8 Exhibition event to earn exclusive rewards! All rewards are untradeable. 1 Of 3 94+ Fof Ptg/Gotg/Gh Team 1 Player Pick Expires in 26 days 5 Objectives 89% 11%</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -17574,12 +17574,12 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Season 8 Exhibition Weekly Play Compete in the Season 8 Exhibition event to earn Coin boost and a consumable item! All rewards are untradeable. Shadow Expires in 27 days 1 Objectives 91% 9%</t>
+          <t>Season 8 Exhibition Weekly Play Compete in the Season 8 Exhibition event to earn Coin boost and a consumable item! All rewards are untradeable. Shadow Expires in 26 days 1 Objectives 91% 9%</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -17611,12 +17611,12 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Season 8 Exhibition Compete in the Season 8 Exhibition event to earn exclusive rewards! All rewards are untradeable. 5X 88+ Rare Gold Players Pack Evo Unlock Expires in 27 days 7 Objectives 90% 10%</t>
+          <t>Season 8 Exhibition Compete in the Season 8 Exhibition event to earn exclusive rewards! All rewards are untradeable. 5X 88+ Rare Gold Players Pack Evo Unlock Expires in 26 days 7 Objectives 90% 10%</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Expires in 27 days</t>
+          <t>Expires in 26 days</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -18568,7 +18568,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Campaign &gt; Path to Glory Week 2 Path to Glory Week 2 - EA SPORTS FC 26 Objectives Complete all the challenges to earn Festival of Football Tokens and SP. All rewards are Untradeable. NEW Path to Glory Week 2 Complete all the challenges to earn Festival of Football Tokens and SP. All rewards are Untradeable. 20 Tokens Expires in 7 days 800 total 5 Objectives 94% 6% Rewards 800 SP 20 Tokens 15 Tokens 10 Tokens 20 Tokens Goal Getter Score a total of 40 goals in any Ultimate Team Game Mode. 20 Tokens Domination Win 4 games by 3 goals or more in Squad Battles matches on min. Semi-Pro Difficulty (or Live Events/Rivals/Champions/Rush). 300 SP Finesse Glory Score 3 goals with a Finesse Shot in any Ultimate Team Game Mode while having at least 4 players from Australia, Uzbekistan, Qatar or New Zealand in your starting 11. 15 Tokens Path to Glory Win 5 matches in any Ultimate Team Game Mode while having at least 1 Path to Glory or National Pride Player Item in your starting 11. 500 SP The Underdogs Win 6 games in any Ultimate Team Game Mode while having at least 1 Player Item from Saudi Arabia, South Korea and Japan in your starting 11. 10 Tokens © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Campaign &gt; Path to Glory Week 2 Path to Glory Week 2 - EA SPORTS FC 26 Objectives Complete all the challenges to earn Festival of Football Tokens and SP. All rewards are Untradeable. NEW Path to Glory Week 2 Complete all the challenges to earn Festival of Football Tokens and SP. All rewards are Untradeable. 20 Tokens Expires in 6 days 800 total 5 Objectives 93% 7% Rewards 800 SP 20 Tokens 15 Tokens 10 Tokens 20 Tokens Goal Getter Score a total of 40 goals in any Ultimate Team Game Mode. 20 Tokens Domination Win 4 games by 3 goals or more in Squad Battles matches on min. Semi-Pro Difficulty (or Live Events/Rivals/Champions/Rush). 300 SP Finesse Glory Score 3 goals with a Finesse Shot in any Ultimate Team Game Mode while having at least 4 players from Australia, Uzbekistan, Qatar or New Zealand in your starting 11. 15 Tokens Path to Glory Win 5 matches in any Ultimate Team Game Mode while having at least 1 Path to Glory or National Pride Player Item in your starting 11. 500 SP The Underdogs Win 6 games in any Ultimate Team Game Mode while having at least 1 Player Item from Saudi Arabia, South Korea and Japan in your starting 11. 10 Tokens © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
     </row>
@@ -18590,7 +18590,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Live Events &gt; Journey of Nations Asia &amp; Oceania Journey of Nations Asia &amp; Oceania - EA SPORTS FC 26 Objectives Compete in the Journey of Nations Asia &amp; Oceania Live Event to earn exclusive rewards! All rewards are untradeable. NEW Journey of Nations Asia &amp; Oceania Compete in the Journey of Nations Asia &amp; Oceania Live Event to earn exclusive rewards! All rewards are untradeable. 87+ Rare Gold Player Pack Expires in 7 days 6 Objectives 87% 13% Rewards Shadow Award Hunter 1x 2x 84+ Rare Gold Players Pack 1x 5x 81+ Rare Gold Players Pack 1x 5x 80+ Rare Gold Players Pack 1x 87+ Rare Gold Player Pack Win 3 Win 3 matches in the Journey of Nations Asia &amp; Oceania Live Event. Shadow Play 3 Play 3 matches in the Journey of Nations Asia &amp; Oceania Live Event. Award Win 2 Win 2 matches in the Journey of Nations Asia &amp; Oceania Live Event. 2X 84+ Rare Gold Players Pack Play 2 Play 2 matches in the Journey of Nations Asia &amp; Oceania Live Event. 5X 81+ Rare Gold Players Pack Win 1 Win 1 match in the Journey of Nations Asia &amp; Oceania Live Event. 5X 80+ Rare Gold Players Pack Play 1 Play 1 match in the Journey of Nations Asia &amp; Oceania Live Event. Hunter © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Live Events &gt; Journey of Nations Asia &amp; Oceania Journey of Nations Asia &amp; Oceania - EA SPORTS FC 26 Objectives Compete in the Journey of Nations Asia &amp; Oceania Live Event to earn exclusive rewards! All rewards are untradeable. NEW Journey of Nations Asia &amp; Oceania Compete in the Journey of Nations Asia &amp; Oceania Live Event to earn exclusive rewards! All rewards are untradeable. 87+ Rare Gold Player Pack Expires in 6 days 6 Objectives 90% 10% Rewards Shadow Award Hunter 1x 2x 84+ Rare Gold Players Pack 1x 5x 81+ Rare Gold Players Pack 1x 5x 80+ Rare Gold Players Pack 1x 87+ Rare Gold Player Pack Win 3 Win 3 matches in the Journey of Nations Asia &amp; Oceania Live Event. Shadow Play 3 Play 3 matches in the Journey of Nations Asia &amp; Oceania Live Event. Award Win 2 Win 2 matches in the Journey of Nations Asia &amp; Oceania Live Event. 2X 84+ Rare Gold Players Pack Play 2 Play 2 matches in the Journey of Nations Asia &amp; Oceania Live Event. 5X 81+ Rare Gold Players Pack Win 1 Win 1 match in the Journey of Nations Asia &amp; Oceania Live Event. 5X 80+ Rare Gold Players Pack Play 1 Play 1 match in the Journey of Nations Asia &amp; Oceania Live Event. Hunter © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
     </row>
@@ -18612,7 +18612,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Campaign &gt; Weekly Rush Points Weekly Rush Points - EA SPORTS FC 26 Objectives Complete Rush Bonuses alongside your teammates to earn Rush Points! Weekly Rush Points Complete Rush Bonuses alongside your teammates to earn Rush Points! 2X 89+ Rare Gold Players Pack 100 Tokens Expires in 6 days 5 Objectives 79% 21% Rewards 100 Tokens 1x 88+ Rare Gold Player Pack 1x 2x 85+ Rare Gold Players Pack 1x 4x 84+ Rare Gold Players Pack 1x 3x 84+ Rare Gold Players Pack 1x 4x 83+ Rare Gold Players Pack 1x 2x 89+ Rare Gold Players Pack 45,000 Rush Points Earn 45,000 points by completing bonuses in Rush. 88+ Rare Gold Player Pack 35,000 Rush Points Earn 35,000 points by completing bonuses in Rush. 2X 85+ Rare Gold Players Pack 25,000 Rush Points Earn 25,000 points by completing bonuses in Rush. 4X 84+ Rare Gold Players Pack 10,000 Rush Points Earn 10,000 points by completing bonuses in Rush. 3X 84+ Rare Gold Players Pack 2,500 Rush Points Earn 2,500 points by completing bonuses in Rush. 4X 83+ Rare Gold Players Pack © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Campaign &gt; Weekly Rush Points Weekly Rush Points - EA SPORTS FC 26 Objectives Complete Rush Bonuses alongside your teammates to earn Rush Points! Weekly Rush Points Complete Rush Bonuses alongside your teammates to earn Rush Points! 2X 89+ Rare Gold Players Pack 100 Tokens Expires in 5 days 5 Objectives 79% 21% Rewards 100 Tokens 1x 88+ Rare Gold Player Pack 1x 2x 85+ Rare Gold Players Pack 1x 4x 84+ Rare Gold Players Pack 1x 3x 84+ Rare Gold Players Pack 1x 4x 83+ Rare Gold Players Pack 1x 2x 89+ Rare Gold Players Pack 45,000 Rush Points Earn 45,000 points by completing bonuses in Rush. 88+ Rare Gold Player Pack 35,000 Rush Points Earn 35,000 points by completing bonuses in Rush. 2X 85+ Rare Gold Players Pack 25,000 Rush Points Earn 25,000 points by completing bonuses in Rush. 4X 84+ Rare Gold Players Pack 10,000 Rush Points Earn 10,000 points by completing bonuses in Rush. 3X 84+ Rare Gold Players Pack 2,500 Rush Points Earn 2,500 points by completing bonuses in Rush. 4X 83+ Rare Gold Players Pack © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
     </row>
@@ -18634,7 +18634,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Seasonal &gt; Season 8 Weekly Play 2 Season 8 Weekly Play 2 - EA SPORTS FC 26 Objectives Complete 3 out of the 5 challenges to earn SP! Season 8 Weekly Play 2 Complete 3 out of the 5 challenges to earn SP! 750 SP Expires in 6 days 2,000 total 3 of 5 Objectives 94% 6% Rewards 2,000 SP Play 5 Live Events Play 5 matches in any Ultimate Team Live Event. 250 SP Play 5 Rush Play 5 Ultimate Team Rush matches. 250 SP Play 5 Champions Play 5 matches in Champions. 250 SP Play 5 Rivals Play 5 matches in Rivals. 250 SP Play 5 Squad Battles Play 5 Squad Battles matches on Min. Semi-Pro difficulty. 250 SP © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Seasonal &gt; Season 8 Weekly Play 2 Season 8 Weekly Play 2 - EA SPORTS FC 26 Objectives Complete 3 out of the 5 challenges to earn SP! Season 8 Weekly Play 2 Complete 3 out of the 5 challenges to earn SP! 750 SP Expires in 5 days 2,000 total 3 of 5 Objectives 94% 6% Rewards 2,000 SP Play 5 Live Events Play 5 matches in any Ultimate Team Live Event. 250 SP Play 5 Rush Play 5 Ultimate Team Rush matches. 250 SP Play 5 Champions Play 5 matches in Champions. 250 SP Play 5 Rivals Play 5 matches in Rivals. 250 SP Play 5 Squad Battles Play 5 Squad Battles matches on Min. Semi-Pro difficulty. 250 SP © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
     </row>
@@ -18656,7 +18656,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Seasonal &gt; Weekly Objectives Weekly Objectives - EA SPORTS FC 26 Objectives Complete weekly Objectives to earn SP! Weekly Objectives Complete weekly Objectives to earn SP! 500 SP Expires in 6 days 1,500 total 5 Objectives 95% 5% Rewards 1,500 SP Score 10 Score 10 goals in any Ultimate Team game mode using a player from Canada. 200 SP Win 10 Win 10 matches in Squad Battles on Min. Semi-Pro difficulty (or Rush/Rivals/Champions/Live Events). 200 SP Play 10 Play 10 matches in Squad Battles on Min. Semi-Pro difficulty (or Rush/Rivals/Champions/Live Events). 200 SP Buy 10 Buy 10 Player Items on the Transfer Market. 200 SP List 10 List 10 Player Items on the Transfer Market. 200 SP © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Seasonal &gt; Weekly Objectives Weekly Objectives - EA SPORTS FC 26 Objectives Complete weekly Objectives to earn SP! Weekly Objectives Complete weekly Objectives to earn SP! 500 SP Expires in 5 days 1,500 total 5 Objectives 96% 4% Rewards 1,500 SP Score 10 Score 10 goals in any Ultimate Team game mode using a player from Canada. 200 SP Win 10 Win 10 matches in Squad Battles on Min. Semi-Pro difficulty (or Rush/Rivals/Champions/Live Events). 200 SP Play 10 Play 10 matches in Squad Battles on Min. Semi-Pro difficulty (or Rush/Rivals/Champions/Live Events). 200 SP Buy 10 Buy 10 Player Items on the Transfer Market. 200 SP List 10 List 10 Player Items on the Transfer Market. 200 SP © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
     </row>
@@ -18678,7 +18678,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Live Events &gt; Path to Glory! Path to Glory! - EA SPORTS FC 26 Objectives Celebrate some of the week's standout international matches in the Path to Glory Live Event with this themed Objective! Earn packs, FOF Tokens, SP, one celebration item, and EVO Rewards. All rewards are untradeable. Path to Glory! Celebrate some of the week's standout international matches in the Path to Glory Live Event with this themed Objective! Earn packs, FOF Tokens, SP, one celebration item, and EVO Rewards. All rewards are untradeable. 170 Tokens Evo Unlock Expires in 2 days 500 total 9 Objectives 86% 14% Rewards 500 SP 90 Tokens Award Evo Unlock 40 Tokens Evo Unlock 170 Tokens Evo Unlock 1x 3x 84+ Rare Gold Players Pack 1x 3x 86+ Rare Gold Players Pack 1x 4x 85+ Rare Gold Players Pack 1x 7x 84+ Rare Gold Players Pack 1x 7x 82+ Rare Gold Players Pack 1x 10x 81+ Rare Gold Players Pack Brazil vs. Morocco Assist 5 goals in the Path to Glory Live Event while having min. 4 players from Brazil or Morocco in your starting 11. 500 SP Qatar vs. Switzerland Win 3 matches in the Path to Glory Live Event while having min. 4 players from Qatar or Switzerland in your starting 11. 90 Tokens 3X 84+ Rare Gold Players Pack Austria vs. Türkiye Score 5 goals in the Path to Glory Live Event while having min. 4 players from Austria or Turkiye in your starting 11. 3X 86+ Rare Gold Players Pack Canada vs. Bosnia and Herzegovina Win 2 matches in the Path to Glory Live Event while having min. 4 players from Canada or Bosnia and Herzegovina in your starting 11. 4X 85+ Rare Gold Players Pack United States vs. Paraguay Play 2 matches in the Path to Glory Live Event while having min. 4 players from USA or Paraguay in your starting 11. 7X 84+ Rare Gold Players Pack Mexico vs. South Africa Score 3 goals in the Path to Glory Live Event while having min. 4 players from Mexico or South Africa in your starting 11. Award South Korea vs. Czechia Score 2 goals with Finesse Shots in the Path to Glory Live Event while having min. 4 players from South Korea or Czechia in your starting 11. Earn an Evo consumable. All EVO details can be previewed. Evo Unlock Score 10 Score 10 goals in the Path to Glory Live Event. 40 Tokens 7X 82+ Rare Gold Players Pack Score 1 Score 1 goal in the Path to Glory Live Event. Earn a Cosmetic EVO. All EVO details can be previewed. Evo Unlock 10X 81+ Rare Gold Players Pack © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Live Events &gt; Path to Glory! Path to Glory! - EA SPORTS FC 26 Objectives Celebrate some of the week's standout international matches in the Path to Glory Live Event with this themed Objective! Earn packs, FOF Tokens, SP, one celebration item, and EVO Rewards. All rewards are untradeable. Path to Glory! Celebrate some of the week's standout international matches in the Path to Glory Live Event with this themed Objective! Earn packs, FOF Tokens, SP, one celebration item, and EVO Rewards. All rewards are untradeable. 170 Tokens Evo Unlock Expires in 23 hours 500 total 9 Objectives 86% 14% Rewards 500 SP 90 Tokens Award Evo Unlock 40 Tokens Evo Unlock 170 Tokens Evo Unlock 1x 3x 84+ Rare Gold Players Pack 1x 3x 86+ Rare Gold Players Pack 1x 4x 85+ Rare Gold Players Pack 1x 7x 84+ Rare Gold Players Pack 1x 7x 82+ Rare Gold Players Pack 1x 10x 81+ Rare Gold Players Pack Brazil vs. Morocco Assist 5 goals in the Path to Glory Live Event while having min. 4 players from Brazil or Morocco in your starting 11. 500 SP Qatar vs. Switzerland Win 3 matches in the Path to Glory Live Event while having min. 4 players from Qatar or Switzerland in your starting 11. 90 Tokens 3X 84+ Rare Gold Players Pack Austria vs. Türkiye Score 5 goals in the Path to Glory Live Event while having min. 4 players from Austria or Turkiye in your starting 11. 3X 86+ Rare Gold Players Pack Canada vs. Bosnia and Herzegovina Win 2 matches in the Path to Glory Live Event while having min. 4 players from Canada or Bosnia and Herzegovina in your starting 11. 4X 85+ Rare Gold Players Pack United States vs. Paraguay Play 2 matches in the Path to Glory Live Event while having min. 4 players from USA or Paraguay in your starting 11. 7X 84+ Rare Gold Players Pack Mexico vs. South Africa Score 3 goals in the Path to Glory Live Event while having min. 4 players from Mexico or South Africa in your starting 11. Award South Korea vs. Czechia Score 2 goals with Finesse Shots in the Path to Glory Live Event while having min. 4 players from South Korea or Czechia in your starting 11. Earn an Evo consumable. All EVO details can be previewed. Evo Unlock Score 10 Score 10 goals in the Path to Glory Live Event. 40 Tokens 7X 82+ Rare Gold Players Pack Score 1 Score 1 goal in the Path to Glory Live Event. Earn a Cosmetic EVO. All EVO details can be previewed. Evo Unlock 10X 81+ Rare Gold Players Pack © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
     </row>
@@ -18700,7 +18700,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Seasonal &gt; Daily Objectives Daily Objectives - EA SPORTS FC 26 Objectives Play, complete, and earn SP from the daily Objective every 24 hours! Daily Objectives Play, complete, and earn SP from the daily Objective every 24 hours! 90 SP Expires in 6 days 190 total 2 Objectives 92% 8% Rewards 190 SP Score 2 goals Score 2 goals in any Ultimate Team game mode. 50 SP Play 1 Play 1 match in any Ultimate Team game mode and earn SP! 50 SP © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Seasonal &gt; Daily Objectives Daily Objectives - EA SPORTS FC 26 Objectives Play, complete, and earn SP from the daily Objective every 24 hours! Daily Objectives Play, complete, and earn SP from the daily Objective every 24 hours! 90 SP Expires in 5 days 190 total 2 Objectives 92% 8% Rewards 190 SP Score 2 goals Score 2 goals in any Ultimate Team game mode. 50 SP Play 1 Play 1 match in any Ultimate Team game mode and earn SP! 50 SP © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
     </row>
@@ -18722,7 +18722,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Seasonal &gt; Season 8 Weekly Play Completionist Season 8 Weekly Play Completionist - EA SPORTS FC 26 Objectives Complete any 4 of the 5 Season 8 Weekly Play Objectives and claim bonus pack rewards. All rewards are untradeable. Season 8 Weekly Play Completionist Complete any 4 of the 5 Season 8 Weekly Play Objectives and claim bonus pack rewards. All rewards are untradeable. Fof Ptg Player Pack Expires in 27 days 4 of 5 Objectives 91% 9% Rewards 1 Of 4 89+ Rare Gold Player Pick 1 Of 4 89+ Rare Gold Player Pick 1x 5x 88+ Rare Gold Players Pack 1x 3x 85+ Rare Gold Players Pack 1x 4x 84+ Rare Gold Players Pack 1x FOF PTG Player Pack Week 5 Complete the Season 8 Weekly Play 5 Objective. 1 Of 4 89+ Rare Gold Player Pick Week 4 Complete the Season 8 Weekly Play 4 Objective. 1 Of 4 89+ Rare Gold Player Pick Week 3 Complete the Season 8 Weekly Play 3 Objective. 5X 88+ Rare Gold Players Pack Week 2 Complete the Season 8 Weekly Play 2 Objective. 3X 85+ Rare Gold Players Pack Week 1 Complete the Season 8 Weekly Play 1 Objective. 4X 84+ Rare Gold Players Pack © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Seasonal &gt; Season 8 Weekly Play Completionist Season 8 Weekly Play Completionist - EA SPORTS FC 26 Objectives Complete any 4 of the 5 Season 8 Weekly Play Objectives and claim bonus pack rewards. All rewards are untradeable. Season 8 Weekly Play Completionist Complete any 4 of the 5 Season 8 Weekly Play Objectives and claim bonus pack rewards. All rewards are untradeable. Fof Ptg Player Pack Expires in 26 days 4 of 5 Objectives 91% 9% Rewards 1 Of 4 89+ Rare Gold Player Pick 1 Of 4 89+ Rare Gold Player Pick 1x 5x 88+ Rare Gold Players Pack 1x 3x 85+ Rare Gold Players Pack 1x 4x 84+ Rare Gold Players Pack 1x FOF PTG Player Pack Week 5 Complete the Season 8 Weekly Play 5 Objective. 1 Of 4 89+ Rare Gold Player Pick Week 4 Complete the Season 8 Weekly Play 4 Objective. 1 Of 4 89+ Rare Gold Player Pick Week 3 Complete the Season 8 Weekly Play 3 Objective. 5X 88+ Rare Gold Players Pack Week 2 Complete the Season 8 Weekly Play 2 Objective. 3X 85+ Rare Gold Players Pack Week 1 Complete the Season 8 Weekly Play 1 Objective. 4X 84+ Rare Gold Players Pack © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
     </row>
@@ -18744,7 +18744,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Live Events &gt; Season 8 Exhibition Weekly Play Completionist Season 8 Exhibition Weekly Play Completionist - EA SPORTS FC 26 Objectives Compete in the Season 8 Exhibition event to earn exclusive rewards! All rewards are untradeable. Season 8 Exhibition Weekly Play Completionist Compete in the Season 8 Exhibition event to earn exclusive rewards! All rewards are untradeable. 1 Of 3 94+ Fof Ptg/Gotg/Gh Team 1 Player Pick Expires in 27 days 5 Objectives 89% 11% Rewards 1 Of 3 Fof Gh Team 1 Player Pick 1 Of 3 Fof Gotg Player Pick 1 Of 3 94+ Fof Ptg/Gotg/Gh Team 1 Player Pick 1x 93+ FOF PTG Team 2 Player Pack 1x 93+ FOF PTG Team 1 Player Pack 1x 5x 87+ Rare Gold Players Pack Week 5 Complete the Season 8 Exhibition Weekly Play Objective 5 times. 1 Of 3 Fof Gh Team 1 Player Pick Week 4 Complete the Season 8 Exhibition Weekly Play Objective 4 times. 1 Of 3 Fof Gotg Player Pick Week 3 Complete the Season 8 Exhibition Weekly Play Objective 3 times. 93+ Fof Ptg Team 2 Player Pack Week 2 Complete the Season 8 Exhibition Weekly Play Objective 2 times. 93+ Fof Ptg Team 1 Player Pack Week 1 Complete the Season 8 Exhibition Weekly Play Objective 1 time. 5X 87+ Rare Gold Players Pack © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Live Events &gt; Season 8 Exhibition Weekly Play Completionist Season 8 Exhibition Weekly Play Completionist - EA SPORTS FC 26 Objectives Compete in the Season 8 Exhibition event to earn exclusive rewards! All rewards are untradeable. Season 8 Exhibition Weekly Play Completionist Compete in the Season 8 Exhibition event to earn exclusive rewards! All rewards are untradeable. 1 Of 3 94+ Fof Ptg/Gotg/Gh Team 1 Player Pick Expires in 26 days 5 Objectives 89% 11% Rewards 1 Of 3 Fof Gh Team 1 Player Pick 1 Of 3 Fof Gotg Player Pick 1 Of 3 94+ Fof Ptg/Gotg/Gh Team 1 Player Pick 1x 93+ FOF PTG Team 2 Player Pack 1x 93+ FOF PTG Team 1 Player Pack 1x 5x 87+ Rare Gold Players Pack Week 5 Complete the Season 8 Exhibition Weekly Play Objective 5 times. 1 Of 3 Fof Gh Team 1 Player Pick Week 4 Complete the Season 8 Exhibition Weekly Play Objective 4 times. 1 Of 3 Fof Gotg Player Pick Week 3 Complete the Season 8 Exhibition Weekly Play Objective 3 times. 93+ Fof Ptg Team 2 Player Pack Week 2 Complete the Season 8 Exhibition Weekly Play Objective 2 times. 93+ Fof Ptg Team 1 Player Pack Week 1 Complete the Season 8 Exhibition Weekly Play Objective 1 time. 5X 87+ Rare Gold Players Pack © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
     </row>
@@ -18766,7 +18766,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Live Events &gt; Season 8 Exhibition Weekly Play Season 8 Exhibition Weekly Play - EA SPORTS FC 26 Objectives Compete in the Season 8 Exhibition event to earn Coin boost and a consumable item! All rewards are untradeable. Season 8 Exhibition Weekly Play Compete in the Season 8 Exhibition event to earn Coin boost and a consumable item! All rewards are untradeable. Shadow Expires in 27 days 1 Objectives 91% 9% Rewards Item Shadow Play 9 Play 9 matches in the Season 8 Exhibition event. Item © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Live Events &gt; Season 8 Exhibition Weekly Play Season 8 Exhibition Weekly Play - EA SPORTS FC 26 Objectives Compete in the Season 8 Exhibition event to earn Coin boost and a consumable item! All rewards are untradeable. Season 8 Exhibition Weekly Play Compete in the Season 8 Exhibition event to earn Coin boost and a consumable item! All rewards are untradeable. Shadow Expires in 26 days 1 Objectives 91% 9% Rewards Item Shadow Play 9 Play 9 matches in the Season 8 Exhibition event. Item © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
     </row>
@@ -18788,7 +18788,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Live Events &gt; Season 8 Exhibition Season 8 Exhibition - EA SPORTS FC 26 Objectives Compete in the Season 8 Exhibition event to earn exclusive rewards! All rewards are untradeable. Season 8 Exhibition Compete in the Season 8 Exhibition event to earn exclusive rewards! All rewards are untradeable. 5X 88+ Rare Gold Players Pack Evo Unlock Expires in 27 days 7 Objectives 90% 10% Rewards Evo Unlock Evo Unlock 1 Of 4 89+ Rare Gold Player Pick 1 Of 4 88+ Rare Gold Players Evo Unlock 1x 10x 87+ Rare Gold Players Pack 1x 5x 87+ Rare Gold Players Pack 1x 3x 88+ Rare Gold Players Pack 1x 5x 88+ Rare Gold Players Pack Score in 30 Score at least 1 goal in 30 separate matches in the Season 8 Exhibition event. Evo Unlock Score in 25 Score at least 1 goal in 25 separate matches in the Season 8 Exhibition event. Evo Unlock Score in 20 Score at least 1 goal in 20 separate matches with a ST in the Season 8 Exhibition event. 10X 87+ Rare Gold Players Pack Assist in 20 Assist at least 1 goal in 20 separate matches with a CM in the Season 8 Exhibition event. 1 Of 4 89+ Rare Gold Player Pick Play 20 Play 20 matches in the Season 8 Exhibition event. 5X 87+ Rare Gold Players Pack Play 10 Play 10 matches in the Season 8 Exhibition event. 1 Of 4 88+ Rare Gold Players Play 5 Play 5 matches in the Season 8 Exhibition event. 3X 88+ Rare Gold Players Pack © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
+          <t>Players SBC Squad Builder Evolutions Objectives Evo Lab GG Club Log In FUT.GG &gt; Objectives &gt; Live Events &gt; Season 8 Exhibition Season 8 Exhibition - EA SPORTS FC 26 Objectives Compete in the Season 8 Exhibition event to earn exclusive rewards! All rewards are untradeable. Season 8 Exhibition Compete in the Season 8 Exhibition event to earn exclusive rewards! All rewards are untradeable. 5X 88+ Rare Gold Players Pack Evo Unlock Expires in 26 days 7 Objectives 90% 10% Rewards Evo Unlock Evo Unlock 1 Of 4 89+ Rare Gold Player Pick 1 Of 4 88+ Rare Gold Players Evo Unlock 1x 10x 87+ Rare Gold Players Pack 1x 5x 87+ Rare Gold Players Pack 1x 3x 88+ Rare Gold Players Pack 1x 5x 88+ Rare Gold Players Pack Score in 30 Score at least 1 goal in 30 separate matches in the Season 8 Exhibition event. Evo Unlock Score in 25 Score at least 1 goal in 25 separate matches in the Season 8 Exhibition event. Evo Unlock Score in 20 Score at least 1 goal in 20 separate matches with a ST in the Season 8 Exhibition event. 10X 87+ Rare Gold Players Pack Assist in 20 Assist at least 1 goal in 20 separate matches with a CM in the Season 8 Exhibition event. 1 Of 4 89+ Rare Gold Player Pick Play 20 Play 20 matches in the Season 8 Exhibition event. 5X 87+ Rare Gold Players Pack Play 10 Play 10 matches in the Season 8 Exhibition event. 1 Of 4 88+ Rare Gold Players Play 5 Play 5 matches in the Season 8 Exhibition event. 3X 88+ Rare Gold Players Pack © 2026 Stormstrike Inc. All rights reserved. Privacy Policy | Terms of Service | Business Inquiries | FIFAIndex | MUT.GG | CFB.FAN | ForzaGarage</t>
         </is>
       </c>
     </row>

</xml_diff>